<commit_message>
Deployed d9f6203e to dev with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/dev/assets/coremeta4cat_vocabulary.xlsx
+++ b/dev/assets/coremeta4cat_vocabulary.xlsx
@@ -5985,7 +5985,7 @@
       <c r="H116" s="13" t="inlineStr"/>
       <c r="I116" s="13" t="inlineStr">
         <is>
-          <t>coremeta4cat:hydrolysis_ratio</t>
+          <t>voc4cat:0008157</t>
         </is>
       </c>
       <c r="J116" s="13" t="inlineStr">
@@ -6113,7 +6113,7 @@
       <c r="H119" s="13" t="inlineStr"/>
       <c r="I119" s="13" t="inlineStr">
         <is>
-          <t>coremeta4cat:surfactant_template</t>
+          <t>voc4cat:0008147</t>
         </is>
       </c>
       <c r="J119" s="13" t="inlineStr">
@@ -6402,7 +6402,7 @@
       </c>
       <c r="I126" s="13" t="inlineStr">
         <is>
-          <t>coremeta4cat:filling_volume</t>
+          <t>voc4cat:0008148</t>
         </is>
       </c>
       <c r="J126" s="13" t="inlineStr">
@@ -6494,7 +6494,7 @@
       <c r="H128" s="13" t="inlineStr"/>
       <c r="I128" s="13" t="inlineStr">
         <is>
-          <t>coremeta4cat:cooling_rate</t>
+          <t>voc4cat:0008149</t>
         </is>
       </c>
       <c r="J128" s="13" t="inlineStr">
@@ -6936,7 +6936,7 @@
       <c r="H139" s="16" t="inlineStr"/>
       <c r="I139" s="16" t="inlineStr">
         <is>
-          <t>coremeta4cat:PlasmaAssisted</t>
+          <t>voc4cat:0008152</t>
         </is>
       </c>
       <c r="J139" s="16" t="inlineStr">
@@ -6981,7 +6981,7 @@
       <c r="H140" s="13" t="inlineStr"/>
       <c r="I140" s="13" t="inlineStr">
         <is>
-          <t>coremeta4cat:plasma_type</t>
+          <t>voc4cat:0008153</t>
         </is>
       </c>
       <c r="J140" s="13" t="inlineStr">
@@ -7029,7 +7029,7 @@
       <c r="H141" s="13" t="inlineStr"/>
       <c r="I141" s="13" t="inlineStr">
         <is>
-          <t>coremeta4cat:power_input</t>
+          <t>voc4cat:0008154</t>
         </is>
       </c>
       <c r="J141" s="13" t="inlineStr">
@@ -7113,7 +7113,7 @@
       <c r="H143" s="13" t="inlineStr"/>
       <c r="I143" s="13" t="inlineStr">
         <is>
-          <t>coremeta4cat:exposure_time</t>
+          <t>voc4cat:0008155</t>
         </is>
       </c>
       <c r="J143" s="13" t="inlineStr">
@@ -7489,7 +7489,7 @@
       <c r="H152" s="16" t="inlineStr"/>
       <c r="I152" s="16" t="inlineStr">
         <is>
-          <t>coremeta4cat:CombustionSynthesis</t>
+          <t>voc4cat:0008156</t>
         </is>
       </c>
       <c r="J152" s="16" t="inlineStr">

</xml_diff>